<commit_message>
Dynamic Weapon Cooldown 번역 갱신
Dynamic Weapon Cooldown - 3038525914
</commit_message>
<xml_diff>
--- a/Data/Dynamic Weapon Cooldown - 3038525914/1.6/Dynamic Weapon Cooldown - 3038525914.xlsx
+++ b/Data/Dynamic Weapon Cooldown - 3038525914/1.6/Dynamic Weapon Cooldown - 3038525914.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\알티\추가\Dynamic Weapon Cooldown - 3038525914\1.6\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zilrt\Documents\Codex\2026-08-20\new-chat-2\outputs\dynamic-weapon-cooldown-ko\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E80F57B-4FFA-4D5E-B984-DEE3E51BD4DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4576C26-9443-456C-A5D3-659C099EB5F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="28800" windowHeight="17985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
   <si>
     <t>Class+Node [(Identifier (Key)]</t>
   </si>
@@ -49,58 +49,40 @@
     <t>ConfigurableDynamicCooldownTitle</t>
   </si>
   <si>
-    <t>Keyed+ConfigurableDynamicCooldown.RangedCooldownManipulationFactor</t>
-  </si>
-  <si>
-    <t>ConfigurableDynamicCooldown.RangedCooldownManipulationFactor</t>
-  </si>
-  <si>
-    <t>Enable ranged manipulation cooldown patch</t>
-  </si>
-  <si>
-    <t>Keyed+ConfigurableDynamicCooldown.RangedCooldownManipulationFactor.Desc</t>
-  </si>
-  <si>
-    <t>ConfigurableDynamicCooldown.RangedCooldownManipulationFactor.Desc</t>
-  </si>
-  <si>
-    <t>If enabled, ranged cooldown is modified by manipulation. (Requires a restart)</t>
-  </si>
-  <si>
-    <t>Keyed+ConfigurableDynamicCooldown.RangedCooldownSightFactor</t>
-  </si>
-  <si>
-    <t>ConfigurableDynamicCooldown.RangedCooldownSightFactor</t>
-  </si>
-  <si>
-    <t>Enable ranged sight cooldown patch</t>
-  </si>
-  <si>
-    <t>Keyed+ConfigurableDynamicCooldown.RangedCooldownSightFactor.Desc</t>
-  </si>
-  <si>
-    <t>ConfigurableDynamicCooldown.RangedCooldownSightFactor.Desc</t>
-  </si>
-  <si>
-    <t>If enabled, ranged cooldown is modified by sight. Unlike manipulation, having sight above 100% has no effect. (Requires a restart)</t>
-  </si>
-  <si>
-    <t>Keyed+ConfigurableDynamicCooldown.MeleeCooldownManipulationFactor</t>
-  </si>
-  <si>
-    <t>ConfigurableDynamicCooldown.MeleeCooldownManipulationFactor</t>
-  </si>
-  <si>
-    <t>Enable melee cooldown patch</t>
-  </si>
-  <si>
-    <t>Keyed+ConfigurableDynamicCooldown.MeleeCooldownManipulationFactor.Desc</t>
-  </si>
-  <si>
-    <t>ConfigurableDynamicCooldown.MeleeCooldownManipulationFactor.Desc</t>
-  </si>
-  <si>
-    <t>If enabled, melee cooldown is modified by manipulation. (Requires a restart)</t>
+    <t>Keyed+ConfigurableDynamicCooldown.RangedCooldownFactor</t>
+  </si>
+  <si>
+    <t>ConfigurableDynamicCooldown.RangedCooldownFactor</t>
+  </si>
+  <si>
+    <t>Ranged Cooldown Patch</t>
+  </si>
+  <si>
+    <t>Keyed+ConfigurableDynamicCooldown.RangedCooldownFactor.Desc</t>
+  </si>
+  <si>
+    <t>ConfigurableDynamicCooldown.RangedCooldownFactor.Desc</t>
+  </si>
+  <si>
+    <t>If enabled, ranged cooldown is modified by manipulation.</t>
+  </si>
+  <si>
+    <t>Keyed+ConfigurableDynamicCooldown.MeleeeCooldownFactor</t>
+  </si>
+  <si>
+    <t>ConfigurableDynamicCooldown.MeleeeCooldownFactor</t>
+  </si>
+  <si>
+    <t>Melee Cooldown Patch</t>
+  </si>
+  <si>
+    <t>Keyed+ConfigurableDynamicCooldown.MeleeeCooldownFactor.Desc</t>
+  </si>
+  <si>
+    <t>ConfigurableDynamicCooldown.MeleeeCooldownFactor.Desc</t>
+  </si>
+  <si>
+    <t>If enabled, melee cooldown is modified by manipulation.</t>
   </si>
   <si>
     <t>Keyed+ConfigurableDynamicCooldown.Scale</t>
@@ -109,7 +91,7 @@
     <t>ConfigurableDynamicCooldown.Scale</t>
   </si>
   <si>
-    <t>Cooldown scale</t>
+    <t>Cooldown Scale</t>
   </si>
   <si>
     <t>Keyed+ConfigurableDynamicCooldown.DiminishingReturns</t>
@@ -118,16 +100,13 @@
     <t>ConfigurableDynamicCooldown.DiminishingReturns</t>
   </si>
   <si>
-    <t>Diminishing returns</t>
-  </si>
-  <si>
     <t>Keyed+ConfigurableDynamicCooldown.MeleeDiminishingReturns</t>
   </si>
   <si>
     <t>ConfigurableDynamicCooldown.MeleeDiminishingReturns</t>
   </si>
   <si>
-    <t>Melee diminishing return rate</t>
+    <t>Melee Diminishing Return Rate</t>
   </si>
   <si>
     <t>Keyed+ConfigurableDynamicCooldown.RangedDiminishingReturns</t>
@@ -136,7 +115,7 @@
     <t>ConfigurableDynamicCooldown.RangedDiminishingReturns</t>
   </si>
   <si>
-    <t>Ranged diminishing return rate</t>
+    <t>Ranged Diminishing Return Rate</t>
   </si>
   <si>
     <t>Keyed+ConfigurableDynamicCooldown.DiminishingReturns.Desc</t>
@@ -145,40 +124,115 @@
     <t>ConfigurableDynamicCooldown.DiminishingReturns.Desc</t>
   </si>
   <si>
-    <t>How much diminshing the cooldown reduction gets after getting higher than 100% manipulation.</t>
-  </si>
-  <si>
-    <t>원거리 조작 능력 재사용 대기시간 패치 활성화</t>
-  </si>
-  <si>
-    <t>활성화하면 원거리 무기의 재사용 대기시간이 조작 능력에 따라 변경됩니다. (재시작 필요)</t>
-  </si>
-  <si>
-    <t>원거리 시력 재사용 대기시간 패치 활성화</t>
-  </si>
-  <si>
-    <t>활성화하면 원거리 무기의 재사용 대기시간이 시력에 따라 변경됩니다. 조작 능력과 달리 시력이 100%를 넘어도 추가 효과는 없습니다. (재시작 필요)</t>
-  </si>
-  <si>
-    <t>근접 재사용 대기시간 패치 활성화</t>
-  </si>
-  <si>
-    <t>활성화하면 근접 공격의 재사용 대기시간이 조작 능력에 따라 변경됩니다. (재시작 필요)</t>
+    <t>How much we begin to diminsh the further beyond 100% manipulation we get.</t>
+  </si>
+  <si>
+    <t>Keyed+ConfigurableDynamicCooldown.CurveMode</t>
+  </si>
+  <si>
+    <t>ConfigurableDynamicCooldown.CurveMode</t>
+  </si>
+  <si>
+    <t>Curve Mode (how manipulation maps to cooldown):</t>
+  </si>
+  <si>
+    <t>Keyed+ConfigurableDynamicCooldown.CurveMode.Diminishing</t>
+  </si>
+  <si>
+    <t>ConfigurableDynamicCooldown.CurveMode.Diminishing</t>
+  </si>
+  <si>
+    <t>Diminishing Returns (default)</t>
+  </si>
+  <si>
+    <t>Keyed+ConfigurableDynamicCooldown.CurveMode.Inverse</t>
+  </si>
+  <si>
+    <t>ConfigurableDynamicCooldown.CurveMode.Inverse</t>
+  </si>
+  <si>
+    <t>Inverse Manipulation (cooldown = 1 / manipulation^strength)</t>
+  </si>
+  <si>
+    <t>Keyed+ConfigurableDynamicCooldown.CurveMode.Linear</t>
+  </si>
+  <si>
+    <t>ConfigurableDynamicCooldown.CurveMode.Linear</t>
+  </si>
+  <si>
+    <t>Linear (no curve)</t>
+  </si>
+  <si>
+    <t>Keyed+ConfigurableDynamicCooldown.InverseInfo</t>
+  </si>
+  <si>
+    <t>ConfigurableDynamicCooldown.InverseInfo</t>
+  </si>
+  <si>
+    <t>Cooldown multiplier = Manipulation^(-strength). At strength 1.0: 100% manipulation = 100% cooldown, 200% = 50%, 500% = 20%, 1000% = 10%. Higher strength rewards manipulation more aggressively.</t>
+  </si>
+  <si>
+    <t>Keyed+ConfigurableDynamicCooldown.RangedInverseStrength</t>
+  </si>
+  <si>
+    <t>ConfigurableDynamicCooldown.RangedInverseStrength</t>
+  </si>
+  <si>
+    <t>Ranged Inverse Strength</t>
+  </si>
+  <si>
+    <t>Keyed+ConfigurableDynamicCooldown.MeleeInverseStrength</t>
+  </si>
+  <si>
+    <t>ConfigurableDynamicCooldown.MeleeInverseStrength</t>
+  </si>
+  <si>
+    <t>Melee Inverse Strength</t>
+  </si>
+  <si>
+    <t>활성화하면 조작 능력에 따라 원거리 공격의 재사용 대기시간이 변경됩니다.</t>
+  </si>
+  <si>
+    <t>근접 재사용 대기시간 패치</t>
+  </si>
+  <si>
+    <t>활성화하면 조작 능력에 따라 근접 공격의 재사용 대기시간이 변경됩니다.</t>
   </si>
   <si>
     <t>재사용 대기시간 배율</t>
   </si>
   <si>
-    <t>점감 효과</t>
-  </si>
-  <si>
-    <t>근접 점감률</t>
-  </si>
-  <si>
-    <t>원거리 점감률</t>
-  </si>
-  <si>
-    <t>조작 능력이 100%를 초과한 뒤 재사용 대기시간 감소 효과가 얼마나 점감되는지를 설정합니다.</t>
+    <t>효과 체감</t>
+  </si>
+  <si>
+    <t>근접 효과 체감률</t>
+  </si>
+  <si>
+    <t>원거리 효과 체감률</t>
+  </si>
+  <si>
+    <t>조작 능력이 100%를 초과할수록 효과를 얼마나 감소시킬지 설정합니다.</t>
+  </si>
+  <si>
+    <t>곡선 모드(조작 능력을 재사용 대기시간에 반영하는 방식):</t>
+  </si>
+  <si>
+    <t>효과 체감(기본값)</t>
+  </si>
+  <si>
+    <t>조작 능력의 역수(재사용 대기시간 = 1 / 조작 능력^강도)</t>
+  </si>
+  <si>
+    <t>선형(곡선 없음)</t>
+  </si>
+  <si>
+    <t>재사용 대기시간 배율 = 조작 능력^(-강도). 강도가 1.0일 때: 조작 능력 100% = 재사용 대기시간 100%, 200% = 50%, 500% = 20%, 1000% = 10%. 강도가 높을수록 높은 조작 능력의 효과가 더욱 커집니다.</t>
+  </si>
+  <si>
+    <t>원거리 역수 강도</t>
+  </si>
+  <si>
+    <t>근접 역수 강도</t>
   </si>
   <si>
     <t>Dynamic Weapon Cooldown</t>
@@ -186,6 +240,80 @@
   </si>
   <si>
     <t>- Dynamic Weapon Cooldown -</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>원거리</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>재사용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>대기시간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>패치</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Diminishing Returns</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -193,7 +321,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -209,6 +337,19 @@
     <font>
       <sz val="8"/>
       <name val="돋움"/>
+      <family val="3"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
     </font>
@@ -236,8 +377,8 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -256,7 +397,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -298,9 +439,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -313,12 +454,52 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="dk1"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="accent1"/>
-        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525">
@@ -376,7 +557,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -402,7 +583,7 @@
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -431,15 +612,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="47.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="58.5703125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="60.5703125" style="1" customWidth="1"/>
+    <col min="1" max="2" width="9.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="31.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="45.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="71.5703125" style="1" customWidth="1"/>
     <col min="7" max="7" width="9.140625" style="1" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
@@ -475,10 +655,10 @@
         <v>8</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -495,7 +675,7 @@
         <v>11</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -511,8 +691,8 @@
       <c r="E4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>43</v>
+      <c r="F4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -528,8 +708,8 @@
       <c r="E5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>44</v>
+      <c r="F5" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -545,8 +725,8 @@
       <c r="E6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>45</v>
+      <c r="F6" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -562,8 +742,8 @@
       <c r="E7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>46</v>
+      <c r="F7" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -577,95 +757,180 @@
         <v>25</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>47</v>
+        <v>74</v>
+      </c>
+      <c r="F8" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>48</v>
+      <c r="F9" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>49</v>
+      <c r="F10" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="1" t="s">
+      <c r="E11" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>50</v>
+      <c r="F11" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>51</v>
+      <c r="F12" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C13" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="F13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="B14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F15" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>52</v>
+      </c>
+      <c r="F17" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F18" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>